<commit_message>
checking sorting algs cheat sheet
</commit_message>
<xml_diff>
--- a/DSA/Sorting/dsa_cheatsheet.xlsx
+++ b/DSA/Sorting/dsa_cheatsheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/balaji.gurusala/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/balaji.gurusala/Documents/Code/coding/DSA/Sorting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B668578-5EC1-0B40-845B-F175C99A3A4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334426BD-E91D-2648-A1BC-93D7190B18F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="27660" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
   <si>
     <t>Algorithm / Concept</t>
   </si>
@@ -46,62 +46,572 @@
     <t>Insertion Sort</t>
   </si>
   <si>
-    <t>Lomuto Partition</t>
-  </si>
-  <si>
-    <t>Hoare Partition</t>
-  </si>
-  <si>
     <t>Brute Force / Incremental</t>
   </si>
   <si>
-    <t>Incremental Shift</t>
-  </si>
-  <si>
-    <t>QuickSort Partitioning</t>
-  </si>
-  <si>
     <t>The Talent Scout: Scan everything ahead, pick absolute minimum, swap to current slot.</t>
   </si>
   <si>
-    <t>The Card Dealer: Take new card, shift larger elements right to clear space, insert card.</t>
-  </si>
-  <si>
-    <t>The Border Patrol: Two pointers move same direction. i tracks border of smaller elements.</t>
-  </si>
-  <si>
     <t>The Pincer Movement: Two pointers move inward from endpoints. Swap outliers until they cross.</t>
   </si>
   <si>
     <t>Outer i is target slot. Inner j scans i+1 to end to find global min index.</t>
   </si>
   <si>
-    <t>Key = arr[i]. While j &gt;= 0 and arr[j] &gt; Key: arr[j+1] = arr[j], then drop key.</t>
-  </si>
-  <si>
-    <t>i = start - 1. j scans start to end-1. If arr[j] &lt; pivot, i++, swap(arr[i], arr[j]).</t>
-  </si>
-  <si>
-    <t>While true: increment left while arr[left] &lt; pivot; decrement right while arr[right] &gt; pivot. If left &gt;= right return right, else swap.</t>
-  </si>
-  <si>
     <t>O(n²) / O(n²) / O(n²)</t>
   </si>
   <si>
     <t>O(n) / O(n²) / O(n²)</t>
   </si>
   <si>
-    <t>O(n) / O(n log n) / O(n²)</t>
-  </si>
-  <si>
     <t>O(1) auxiliary</t>
+  </si>
+  <si>
+    <r>
+      <t>The Right Wall:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>Heavy elements sink right. Each pass guarantees the max unsorted element lands at the far right</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Outer </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>i</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tracks completed passes. Inner </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>j</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> always starts at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and shrinks on the right via </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>len(A) - 1 - i</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to avoid the sorted wall.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>O(n)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>O(n²)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>O(n²)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Best case is O(n) only with early stop flag i.e swapped = True or not)</t>
+    </r>
+  </si>
+  <si>
+    <t>Bubble Sort 
+(large element to right)</t>
+  </si>
+  <si>
+    <t>Bubble Sort
+(Small element to left)</t>
+  </si>
+  <si>
+    <r>
+      <t>The Rising Bubble:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>Light elements float left. Moving from right to left, adjacent pairs are swapped, locking the absolute minimum at the front left wall.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Outer </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>i</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> marks the left wall boundary (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>len(A)-1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">). Inner </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>j</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> moves backward from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>len(A)-1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> down to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>i+1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, comparing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>A[j]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>A[j-1]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Incremental Shift/
+Incremental / Decrease &amp; Conquer</t>
+  </si>
+  <si>
+    <t>The Card Dealer: Take new card, shift larger elements right to clear space, insert card. or
+Shifting Furniture: Lift current item up (key = A[i]) leaving a virtual hole. Slide larger items right until the gap is found, then drop the item down.</t>
+  </si>
+  <si>
+    <t>Key = arr[i]. While j &gt;= 0 and arr[j] &gt; Key: arr[j+1] = arr[j], then drop key. Or
+Outer i lifts key starting at index 1. Inner decrements while j &gt;= 1 and A[j-1] &gt; key. Overwrites A[j] = A[j-1] to slide elements, then drops key into final A[j].</t>
+  </si>
+  <si>
+    <t>Recursive Insertion Sort (Top-Down)</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer (Decrease by 1) / Call Stack Automation</t>
+  </si>
+  <si>
+    <t>The Unwinding Hand: Deal all cards out into space until you hold just 1 card. Re-collect cards one-by-one on the way back, shifting larger cards right to slot each back in.</t>
+  </si>
+  <si>
+    <t>Base case: size &lt;= 1 returns. Recurse downward on size-1. Unwinding: Set key = A[size-1], track hole with j = size-1. While j &gt;= 1 and A[j-1] &gt; key, slide right and decrement j. Drop key into A[j].</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O(n)  / O(n²)  / O(n²) </t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer / Two-Pointer Merge</t>
+  </si>
+  <si>
+    <t>Merge Sort (Recursive)</t>
+  </si>
+  <si>
+    <t>The Converted Zipper: Rip a line of items cleanly down the center recursively until single elements remain. Then zip adjacent pairs back together in perfect sorted order.</t>
+  </si>
+  <si>
+    <t>Helper: mid = start + (end-start)//2. Recurse left and right, then merge. Merge: Two pointers track left half (i=start to mid) and right half (j=mid+1 to end). Compare and append smaller to temp array B, then copy B back into A[start...end].</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O(n log n)  / O(n log n)  / O(n log n) </t>
+  </si>
+  <si>
+    <t>QuickSort (Lomuto)</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer / Recursive Partitioning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O(n log n)  / O(n log n)  / O(n²) </t>
+  </si>
+  <si>
+    <t>O(log n) average auxiliary space / O(n) worst-case space (due to the recursive call stack depth)</t>
+  </si>
+  <si>
+    <t>Base case: if start &gt;= end, return. Partition: smaller = start. For bigger from start + 1 to end: if arr[bigger] &lt;= pivot, smaller++,  swap(arr[smaller], arr[bigger]). Final partition step: swap(arr[smaller], arr[start]). Recurse on QuickSort(start, smaller-1) and QuickSort(smaller+1, end).</t>
+  </si>
+  <si>
+    <r>
+      <t>The Border Patrol Framework: Choose a pivot and copy to starting position. Use a fast scanner (bigger</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>and a slow border pointer (smaller). Push all small elements behind the border, swap the pivot into final border place, and recursively sort the left and right halves.</t>
+    </r>
+  </si>
+  <si>
+    <t>QuickSort (Unified Pincer Hoare)</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer / Safe Converging Pincer</t>
+  </si>
+  <si>
+    <t>Base case: if start &gt;= end, return. Partition: left = start-1, right = end+1. Outer while True. Inner loops: left += 1 until arr[left] &gt;= pivot; right -= 1 until arr[right] &lt;= pivot. If left &gt;= right, return split_index = right. Else, swap(arr[left], arr[right]). Recurse on QuickSort(start, split_index) and QuickSort(split_index+1, end).</t>
+  </si>
+  <si>
+    <t>O(log n) average auxiliary space / O(n) worst-case space</t>
+  </si>
+  <si>
+    <t>O(n) worst-case space (due to the recursive call stack depth)</t>
+  </si>
+  <si>
+    <t>O(n) auxiliary space</t>
+  </si>
+  <si>
+    <t>QuickSort (Hoare)</t>
+  </si>
+  <si>
+    <t>Divide &amp; Conquer / Converging Pincer Partitioning</t>
+  </si>
+  <si>
+    <t>The Inward Pincer Framework: Choose a pivot (typically the start). Two pointers march inward from both endpoints simultaneously. Swap out-of-place pairs until they cross, then recursively split and sort the two resulting blocks.</t>
+  </si>
+  <si>
+    <t>Base case: if start &gt;= end, return. Partition: left = start+1, right = end. Loop: left++ while arr[left] &lt; pivot; right-- while arr[right] &gt; pivot. If left &gt;= right, return split_index = right. Recurse on QuickSort(start, split_index-1) and QuickSort(split_index+1, end).</t>
+  </si>
+  <si>
+    <t>O(n logn) / O(n log n) / O(n²)</t>
+  </si>
+  <si>
+    <t>Counting Sort</t>
+  </si>
+  <si>
+    <t>Non-Comparison Based / Frequency Hashing</t>
+  </si>
+  <si>
+    <t>The Post Office Boxes: Create a labeled bucket for every possible number from 0 to MAX. Walk down your list and drop a tally mark into the matching bucket. Empty the buckets in order to reconstruct the sorted list.</t>
+  </si>
+  <si>
+    <t>1. Initialize max = 0. Loop i in range(0, len(A)) to find global max. 2. Initialize Aux frequency array of size max + 1. 3. Populate: Loop j in range(0, len(A)) and increment Aux[A[j]] += 1. 4. Reconstruct: Loop index k from 0 to max, check if count exists, and overwrite into original array sequentially.</t>
+  </si>
+  <si>
+    <t>O(n + k) auxiliary space</t>
+  </si>
+  <si>
+    <t>O(k + n)  / O(k + n)  / O(k + n)   
+(where k is the maximum element range)</t>
+  </si>
+  <si>
+    <t>Two Sum (Brute Force)</t>
+  </si>
+  <si>
+    <t>Brute Force / Nested Iteration</t>
+  </si>
+  <si>
+    <t>The Blind Pairer: Pick up the first element. Scan every single element ahead of it to check for a match. If no match, drop it, pick up the second element, and repeat the entire scan.</t>
+  </si>
+  <si>
+    <t>Outer loop i from 0 to N-2. Inner loop j from i+1 to N-1. Check if arr[i] + arr[j] == target. Returns indices [i, j]. No sorting required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O(n²)  / O(n²)  / O(n²) </t>
+  </si>
+  <si>
+    <t>Two Sum (Two-Pointer Method)</t>
+  </si>
+  <si>
+    <t>Array Sorting / Converging Pincer Movement</t>
+  </si>
+  <si>
+    <t>The Tug-of-War: Put left and right pointers at both ends of a sorted line. If the current sum is too small, pull the left hand inward to increase it. If the sum is too big, pull the right hand inward to decrease it.</t>
+  </si>
+  <si>
+    <t>Requires array to be sorted first. Initialize left = 0, right = N-1. While left &lt; right: calculate sum = arr[left] + arr[right]. If sum == target, return values/indices. If sum &lt; target, left++. Else, right--.</t>
+  </si>
+  <si>
+    <t>O(n log n) best / O(n log n) average / O(n log n) worst (Dominated completely by the initial sorting step; pointer scan alone is O(n))</t>
+  </si>
+  <si>
+    <t>O(1) auxiliary to O(n) space (Depends entirely on the space complexity of the sorting algorithm used)</t>
+  </si>
+  <si>
+    <t>Two Sum (Hash Map Method)</t>
+  </si>
+  <si>
+    <t>Space-Time Trade-off / Complement Lookup Table</t>
+  </si>
+  <si>
+    <t>The Coat Check: As you walk past an item, calculate exactly what partner item is needed to hit the target (complement = target - current). Look at your storage rack; if the complement is already there, you found your match. If not, hang your current item on the rack and keep moving.</t>
+  </si>
+  <si>
+    <t>Initialize empty map/dictionary {value: index}. Loop i from 0 to N-1. Calculate complement = target - arr[i]. If complement in map, return [map[complement], i]. Else, insert map[arr[i]] = i.</t>
+  </si>
+  <si>
+    <t>O(n) auxiliary space (Worst case stores N-1 elements in the hash map dictionary)</t>
+  </si>
+  <si>
+    <t>O(1) best / O(n) average / O(n) worst (Amortized linear time due to O(1) hash map lookups)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -111,11 +621,49 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -153,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -161,8 +709,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -468,14 +1020,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="28.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="28.6640625" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="56.5" style="3" customWidth="1"/>
-    <col min="4" max="4" width="58.1640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="44.83203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="41.33203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="56.5" style="4" customWidth="1"/>
+    <col min="4" max="4" width="58.1640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="41.33203125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="35.83203125" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="28.6640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,88 +1048,268 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:6" ht="69" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="92" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="44" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="88" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="154" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
+      <c r="D9" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
+    <row r="10" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="88" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="4" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
+    <row r="13" spans="1:6" ht="110" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
-        <v>24</v>
+    <row r="14" spans="1:6" ht="132" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>